<commit_message>
Account for challenge fees and add Profit column to reports
monthly_report.py now emits a PURCHASE event for the initial account
plus every loss replacement, charging CHALLENGE_FEE (default $549,
FundingPips 2 standard $100K). Each month's stats grow two new
fields - challenges_count and fees_sum - and a derived Profit =
Payouts $ - Fees $.

Excel exporter mirrors the new columns on both Monthly and Yearly
sheets. Profit cells render green when positive, red when negative
so the late-period regime change is obvious at a glance.

Run totals over the 2018-12 -> 2026-05 backtest:
  Accounts purchased: 203 (1 initial + 202 replacements)
  Payouts: 1,298 ($5,737,350)
  Fees:    $111,447
  Net profit: $5,625,903

https://claude.ai/code/session_01SXbENjEfxHT3GywVfWjfzo
</commit_message>
<xml_diff>
--- a/reports/monthly_payouts.xlsx
+++ b/reports/monthly_payouts.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Yearly" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monthly'!$A$1:$F$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Yearly'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monthly'!$A$1:$I$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Yearly'!$A$1:$I$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,12 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <color rgb="00007A00"/>
+    </font>
+    <font>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -83,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -94,11 +100,20 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -466,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -475,6 +490,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,6 +526,21 @@
           <t>Payouts $</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Challenges #</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fees $</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Profit $</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -530,6 +563,15 @@
       <c r="F2" s="3" t="n">
         <v>12707.71</v>
       </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>12158.71</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -552,6 +594,15 @@
       <c r="F3" s="3" t="n">
         <v>12960.47</v>
       </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>12960.47</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -574,6 +625,15 @@
       <c r="F4" s="3" t="n">
         <v>22060.51</v>
       </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>22060.51</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -596,6 +656,15 @@
       <c r="F5" s="3" t="n">
         <v>17911.43</v>
       </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>17911.43</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -618,6 +687,15 @@
       <c r="F6" s="3" t="n">
         <v>16403</v>
       </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>16403</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -640,6 +718,15 @@
       <c r="F7" s="3" t="n">
         <v>45082.68</v>
       </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>45082.68</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -662,6 +749,15 @@
       <c r="F8" s="3" t="n">
         <v>37507.27</v>
       </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>37507.27</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -684,6 +780,15 @@
       <c r="F9" s="3" t="n">
         <v>26047</v>
       </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>26047</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -706,6 +811,15 @@
       <c r="F10" s="3" t="n">
         <v>56094.84</v>
       </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>56094.84</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -728,6 +842,15 @@
       <c r="F11" s="3" t="n">
         <v>38310.63</v>
       </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>38310.63</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -750,6 +873,15 @@
       <c r="F12" s="3" t="n">
         <v>38456</v>
       </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>38456</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -772,6 +904,15 @@
       <c r="F13" s="3" t="n">
         <v>20589</v>
       </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>20589</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -794,6 +935,15 @@
       <c r="F14" s="3" t="n">
         <v>16212</v>
       </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>16212</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -816,6 +966,15 @@
       <c r="F15" s="3" t="n">
         <v>24538</v>
       </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>24538</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -838,6 +997,15 @@
       <c r="F16" s="3" t="n">
         <v>77802.82000000001</v>
       </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>77802.82000000001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -860,6 +1028,15 @@
       <c r="F17" s="3" t="n">
         <v>193827.1</v>
       </c>
+      <c r="G17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>192729.1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -882,6 +1059,15 @@
       <c r="F18" s="3" t="n">
         <v>85581</v>
       </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>85581</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -904,6 +1090,15 @@
       <c r="F19" s="3" t="n">
         <v>80640</v>
       </c>
+      <c r="G19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>80640</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -926,6 +1121,15 @@
       <c r="F20" s="3" t="n">
         <v>98228</v>
       </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>98228</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -948,6 +1152,15 @@
       <c r="F21" s="3" t="n">
         <v>80838</v>
       </c>
+      <c r="G21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>80838</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -970,6 +1183,15 @@
       <c r="F22" s="3" t="n">
         <v>50436</v>
       </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>50436</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -992,6 +1214,15 @@
       <c r="F23" s="3" t="n">
         <v>140019</v>
       </c>
+      <c r="G23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>140019</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1014,6 +1245,15 @@
       <c r="F24" s="3" t="n">
         <v>113578</v>
       </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>113578</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1036,6 +1276,15 @@
       <c r="F25" s="3" t="n">
         <v>129994</v>
       </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>129994</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1058,6 +1307,15 @@
       <c r="F26" s="3" t="n">
         <v>50046</v>
       </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>50046</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1080,6 +1338,15 @@
       <c r="F27" s="3" t="n">
         <v>79276</v>
       </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>79276</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1102,6 +1369,15 @@
       <c r="F28" s="3" t="n">
         <v>75765</v>
       </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>75765</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1124,6 +1400,15 @@
       <c r="F29" s="3" t="n">
         <v>149589</v>
       </c>
+      <c r="G29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>149040</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1146,6 +1431,15 @@
       <c r="F30" s="3" t="n">
         <v>85279</v>
       </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>85279</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1168,6 +1462,15 @@
       <c r="F31" s="3" t="n">
         <v>88027</v>
       </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>88027</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1190,6 +1493,15 @@
       <c r="F32" s="3" t="n">
         <v>84814</v>
       </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>84814</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1212,6 +1524,15 @@
       <c r="F33" s="3" t="n">
         <v>68196</v>
       </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>68196</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1234,6 +1555,15 @@
       <c r="F34" s="3" t="n">
         <v>73223</v>
       </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>73223</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1256,6 +1586,15 @@
       <c r="F35" s="3" t="n">
         <v>77128</v>
       </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>77128</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1278,6 +1617,15 @@
       <c r="F36" s="3" t="n">
         <v>89774</v>
       </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>89774</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1300,6 +1648,15 @@
       <c r="F37" s="3" t="n">
         <v>99454</v>
       </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>99454</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1322,6 +1679,15 @@
       <c r="F38" s="3" t="n">
         <v>133865</v>
       </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>133865</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1344,6 +1710,15 @@
       <c r="F39" s="3" t="n">
         <v>195101</v>
       </c>
+      <c r="G39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>194552</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1366,6 +1741,15 @@
       <c r="F40" s="3" t="n">
         <v>181972</v>
       </c>
+      <c r="G40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>181423</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1388,6 +1772,15 @@
       <c r="F41" s="3" t="n">
         <v>197812</v>
       </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>197812</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1410,6 +1803,15 @@
       <c r="F42" s="3" t="n">
         <v>149860</v>
       </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>149860</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1432,6 +1834,15 @@
       <c r="F43" s="3" t="n">
         <v>242656</v>
       </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>242656</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1454,6 +1865,15 @@
       <c r="F44" s="3" t="n">
         <v>174217</v>
       </c>
+      <c r="G44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>173668</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1476,6 +1896,15 @@
       <c r="F45" s="3" t="n">
         <v>114425</v>
       </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>114425</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1498,6 +1927,15 @@
       <c r="F46" s="3" t="n">
         <v>123659</v>
       </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>123659</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1520,6 +1958,15 @@
       <c r="F47" s="3" t="n">
         <v>138425</v>
       </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>138425</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1542,6 +1989,15 @@
       <c r="F48" s="3" t="n">
         <v>172189</v>
       </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>172189</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1564,6 +2020,15 @@
       <c r="F49" s="3" t="n">
         <v>135073</v>
       </c>
+      <c r="G49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>135073</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1586,6 +2051,15 @@
       <c r="F50" s="3" t="n">
         <v>98789</v>
       </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>98789</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1608,6 +2082,15 @@
       <c r="F51" s="3" t="n">
         <v>81974</v>
       </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>81974</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1630,6 +2113,15 @@
       <c r="F52" s="3" t="n">
         <v>89952</v>
       </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>89952</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1652,6 +2144,15 @@
       <c r="F53" s="3" t="n">
         <v>135726</v>
       </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>135726</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1674,6 +2175,15 @@
       <c r="F54" s="3" t="n">
         <v>84524</v>
       </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>84524</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1696,6 +2206,15 @@
       <c r="F55" s="3" t="n">
         <v>80573</v>
       </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>80573</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1718,6 +2237,15 @@
       <c r="F56" s="3" t="n">
         <v>74948</v>
       </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>74948</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1740,6 +2268,15 @@
       <c r="F57" s="3" t="n">
         <v>43003</v>
       </c>
+      <c r="G57" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>41905</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1762,6 +2299,15 @@
       <c r="F58" s="3" t="n">
         <v>43606</v>
       </c>
+      <c r="G58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>43057</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1784,6 +2330,15 @@
       <c r="F59" s="3" t="n">
         <v>8239</v>
       </c>
+      <c r="G59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>7141</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1806,6 +2361,15 @@
       <c r="F60" s="3" t="n">
         <v>25007</v>
       </c>
+      <c r="G60" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>2196</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>22811</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1828,6 +2392,15 @@
       <c r="F61" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G61" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>3294</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>-3294</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1850,6 +2423,15 @@
       <c r="F62" s="3" t="n">
         <v>4276</v>
       </c>
+      <c r="G62" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>1647</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>2629</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1872,6 +2454,15 @@
       <c r="F63" s="3" t="n">
         <v>4303</v>
       </c>
+      <c r="G63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>3205</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1894,6 +2485,15 @@
       <c r="F64" s="3" t="n">
         <v>16327</v>
       </c>
+      <c r="G64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>15229</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1916,6 +2516,15 @@
       <c r="F65" s="3" t="n">
         <v>44836</v>
       </c>
+      <c r="G65" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>43738</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1938,6 +2547,15 @@
       <c r="F66" s="3" t="n">
         <v>8513</v>
       </c>
+      <c r="G66" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>1647</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>6866</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1960,6 +2578,15 @@
       <c r="F67" s="3" t="n">
         <v>13826</v>
       </c>
+      <c r="G67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>12728</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1982,6 +2609,15 @@
       <c r="F68" s="3" t="n">
         <v>4076</v>
       </c>
+      <c r="G68" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>2745</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>1331</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2004,6 +2640,15 @@
       <c r="F69" s="3" t="n">
         <v>41085</v>
       </c>
+      <c r="G69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>1647</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>39438</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2026,6 +2671,15 @@
       <c r="F70" s="3" t="n">
         <v>103582</v>
       </c>
+      <c r="G70" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>2196</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>101386</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2048,6 +2702,15 @@
       <c r="F71" s="3" t="n">
         <v>58200</v>
       </c>
+      <c r="G71" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>1647</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>56553</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2070,6 +2733,15 @@
       <c r="F72" s="3" t="n">
         <v>30505</v>
       </c>
+      <c r="G72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>29956</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2092,6 +2764,15 @@
       <c r="F73" s="3" t="n">
         <v>21119</v>
       </c>
+      <c r="G73" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>1647</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>19472</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2114,6 +2795,15 @@
       <c r="F74" s="3" t="n">
         <v>14787</v>
       </c>
+      <c r="G74" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H74" s="3" t="n">
+        <v>2196</v>
+      </c>
+      <c r="I74" s="4" t="n">
+        <v>12591</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2136,6 +2826,15 @@
       <c r="F75" s="3" t="n">
         <v>65491</v>
       </c>
+      <c r="G75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H75" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I75" s="4" t="n">
+        <v>64393</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2158,6 +2857,15 @@
       <c r="F76" s="3" t="n">
         <v>32402</v>
       </c>
+      <c r="G76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I76" s="4" t="n">
+        <v>31853</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2180,6 +2888,15 @@
       <c r="F77" s="3" t="n">
         <v>82888</v>
       </c>
+      <c r="G77" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>3294</v>
+      </c>
+      <c r="I77" s="4" t="n">
+        <v>79594</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2202,6 +2919,15 @@
       <c r="F78" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G78" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H78" s="3" t="n">
+        <v>4941</v>
+      </c>
+      <c r="I78" s="5" t="n">
+        <v>-4941</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2224,6 +2950,15 @@
       <c r="F79" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G79" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H79" s="3" t="n">
+        <v>3294</v>
+      </c>
+      <c r="I79" s="5" t="n">
+        <v>-3294</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2246,6 +2981,15 @@
       <c r="F80" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G80" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H80" s="3" t="n">
+        <v>3843</v>
+      </c>
+      <c r="I80" s="5" t="n">
+        <v>-3843</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2268,6 +3012,15 @@
       <c r="F81" s="3" t="n">
         <v>4530</v>
       </c>
+      <c r="G81" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H81" s="3" t="n">
+        <v>3294</v>
+      </c>
+      <c r="I81" s="4" t="n">
+        <v>1236</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2290,6 +3043,15 @@
       <c r="F82" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G82" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H82" s="3" t="n">
+        <v>4392</v>
+      </c>
+      <c r="I82" s="5" t="n">
+        <v>-4392</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2312,6 +3074,15 @@
       <c r="F83" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G83" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H83" s="3" t="n">
+        <v>2745</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>-2745</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2334,6 +3105,15 @@
       <c r="F84" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G84" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>5490</v>
+      </c>
+      <c r="I84" s="5" t="n">
+        <v>-5490</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2356,6 +3136,15 @@
       <c r="F85" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G85" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>9333</v>
+      </c>
+      <c r="I85" s="5" t="n">
+        <v>-9333</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2378,6 +3167,15 @@
       <c r="F86" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G86" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>9333</v>
+      </c>
+      <c r="I86" s="5" t="n">
+        <v>-9333</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2400,6 +3198,15 @@
       <c r="F87" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G87" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="I87" s="5" t="n">
+        <v>-6039</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2422,6 +3229,15 @@
       <c r="F88" s="3" t="n">
         <v>4614</v>
       </c>
+      <c r="G88" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>7686</v>
+      </c>
+      <c r="I88" s="5" t="n">
+        <v>-3072</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2444,6 +3260,15 @@
       <c r="F89" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G89" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>7686</v>
+      </c>
+      <c r="I89" s="5" t="n">
+        <v>-7686</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2466,6 +3291,15 @@
       <c r="F90" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G90" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>5490</v>
+      </c>
+      <c r="I90" s="5" t="n">
+        <v>-5490</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2488,31 +3322,49 @@
       <c r="F91" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="G91" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I91" s="5" t="n">
+        <v>-549</v>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+      <c r="A92" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B92" s="5" t="n">
+      <c r="B92" s="7" t="n">
         <v>77</v>
       </c>
-      <c r="C92" s="5" t="n">
+      <c r="C92" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="D92" s="5" t="n">
+      <c r="D92" s="7" t="n">
         <v>202</v>
       </c>
-      <c r="E92" s="5" t="n">
+      <c r="E92" s="7" t="n">
         <v>1298</v>
       </c>
-      <c r="F92" s="6" t="n">
+      <c r="F92" s="8" t="n">
         <v>5737350.46</v>
       </c>
+      <c r="G92" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="H92" s="8" t="n">
+        <v>111447</v>
+      </c>
+      <c r="I92" s="9" t="n">
+        <v>5625903.46</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F91"/>
+  <autoFilter ref="A1:I91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2523,7 +3375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2532,6 +3384,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2565,6 +3420,21 @@
           <t>Payouts $</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Challenges #</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fees $</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Profit $</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2587,6 +3457,15 @@
       <c r="F2" s="3" t="n">
         <v>12707.71</v>
       </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>12158.71</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2609,6 +3488,15 @@
       <c r="F3" s="3" t="n">
         <v>347634.83</v>
       </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>347634.83</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2631,6 +3519,15 @@
       <c r="F4" s="3" t="n">
         <v>1125527.92</v>
       </c>
+      <c r="G4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1098</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1124429.92</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2653,6 +3550,15 @@
       <c r="F5" s="3" t="n">
         <v>1104390</v>
       </c>
+      <c r="G5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>549</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>1103841</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2675,6 +3581,15 @@
       <c r="F6" s="3" t="n">
         <v>1924178</v>
       </c>
+      <c r="G6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>1647</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1922531</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2697,6 +3612,15 @@
       <c r="F7" s="3" t="n">
         <v>671828</v>
       </c>
+      <c r="G7" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>9882</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>661946</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2719,6 +3643,15 @@
       <c r="F8" s="3" t="n">
         <v>361159</v>
       </c>
+      <c r="G8" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>18666</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>342493</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2741,6 +3674,15 @@
       <c r="F9" s="3" t="n">
         <v>185311</v>
       </c>
+      <c r="G9" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>51606</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>133705</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2763,31 +3705,49 @@
       <c r="F10" s="3" t="n">
         <v>4614</v>
       </c>
+      <c r="G10" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>27450</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>-22836</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="7" t="n">
         <v>77</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="7" t="n">
         <v>202</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="7" t="n">
         <v>1298</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="8" t="n">
         <v>5737350.46</v>
       </c>
+      <c r="G11" s="7" t="n">
+        <v>203</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>111447</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>5625903.46</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F10"/>
+  <autoFilter ref="A1:I10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>